<commit_message>
feat: migrate reports and sync workflow to SQLite app
</commit_message>
<xml_diff>
--- a/data/BasketAranjuez/stats_basket_aranjuez_vs_valcude_30-11-25.xlsx
+++ b/data/BasketAranjuez/stats_basket_aranjuez_vs_valcude_30-11-25.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\PyCharm\feb_scraper\data\BasketAranjuez\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE7F888F-B2AA-48FA-942A-C6C0455EC3B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBB10337-FE89-47D8-A27F-754A1051C75A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="30612" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{A3DF5DE4-86F4-4941-B67B-7F07D8A7C005}"/>
   </bookViews>
@@ -218,9 +218,6 @@
     <t>10</t>
   </si>
   <si>
-    <t>Jorge Marcos</t>
-  </si>
-  <si>
     <t>04:58</t>
   </si>
   <si>
@@ -396,6 +393,9 @@
   </si>
   <si>
     <t>Valcude</t>
+  </si>
+  <si>
+    <t>Jorge</t>
   </si>
 </sst>
 </file>
@@ -1191,10 +1191,10 @@
         <v>56</v>
       </c>
       <c r="B5" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>57</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>58</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>33</v>
@@ -1277,13 +1277,13 @@
     </row>
     <row r="6" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="2" t="s">
         <v>60</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>61</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>50</v>
@@ -1295,7 +1295,7 @@
         <v>45</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="H6" s="2" t="s">
         <v>30</v>
@@ -1313,7 +1313,7 @@
         <v>40</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="N6" s="2" t="s">
         <v>29</v>
@@ -1361,40 +1361,40 @@
         <v>40</v>
       </c>
       <c r="AC6" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="7" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="B7" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="C7" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="C7" s="5" t="s">
-        <v>67</v>
-      </c>
       <c r="D7" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E7" s="5" t="s">
         <v>33</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G7" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="J7" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="H7" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="I7" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="J7" s="5" t="s">
-        <v>69</v>
-      </c>
       <c r="K7" s="5" t="s">
         <v>37</v>
       </c>
@@ -1402,7 +1402,7 @@
         <v>36</v>
       </c>
       <c r="M7" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="N7" s="5" t="s">
         <v>36</v>
@@ -1450,18 +1450,18 @@
         <v>46</v>
       </c>
       <c r="AC7" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="8" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="C8" s="2" t="s">
         <v>72</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>73</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>46</v>
@@ -1473,7 +1473,7 @@
         <v>38</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H8" s="2" t="s">
         <v>30</v>
@@ -1491,7 +1491,7 @@
         <v>38</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="N8" s="2" t="s">
         <v>36</v>
@@ -1533,10 +1533,10 @@
         <v>36</v>
       </c>
       <c r="AA8" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="AB8" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="AC8" s="3" t="s">
         <v>46</v>
@@ -1544,14 +1544,14 @@
     </row>
     <row r="9" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="B9" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="C9" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="C9" s="5" t="s">
-        <v>77</v>
-      </c>
       <c r="D9" s="5" t="s">
         <v>36</v>
       </c>
@@ -1562,7 +1562,7 @@
         <v>36</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="H9" s="5" t="s">
         <v>30</v>
@@ -1633,13 +1633,13 @@
     </row>
     <row r="10" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="C10" s="2" t="s">
         <v>79</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>80</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>29</v>
@@ -1722,13 +1722,13 @@
     </row>
     <row r="11" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="B11" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="C11" s="5" t="s">
         <v>82</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>83</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>45</v>
@@ -1749,7 +1749,7 @@
         <v>40</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K11" s="5" t="s">
         <v>30</v>
@@ -1811,13 +1811,13 @@
     </row>
     <row r="12" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="C12" s="2" t="s">
         <v>85</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>86</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>42</v>
@@ -1865,7 +1865,7 @@
         <v>33</v>
       </c>
       <c r="S12" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="T12" s="2" t="s">
         <v>29</v>
@@ -1889,13 +1889,13 @@
         <v>36</v>
       </c>
       <c r="AA12" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="AB12" s="2" t="s">
         <v>49</v>
       </c>
       <c r="AC12" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>
@@ -1910,27 +1910,27 @@
   <sheetData>
     <row r="1" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="B1" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="C1" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="D1" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="E1" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="E1" s="7" t="s">
-        <v>114</v>
-      </c>
       <c r="F1" s="7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="2" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B2" s="7">
         <v>13</v>
@@ -1950,7 +1950,7 @@
     </row>
     <row r="3" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B3" s="7">
         <v>9</v>
@@ -1970,13 +1970,13 @@
     </row>
     <row r="6" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="C6" s="7" t="s">
         <v>115</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>110</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="7" spans="1:35" x14ac:dyDescent="0.3">
@@ -2081,67 +2081,67 @@
     </row>
     <row r="9" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B9" s="8" t="s">
         <v>12</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="J9" s="5" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="K9" s="5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="L9" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="M9" s="5" t="s">
         <v>94</v>
-      </c>
-      <c r="M9" s="5" t="s">
-        <v>95</v>
       </c>
       <c r="N9" s="5" t="s">
         <v>45</v>
       </c>
       <c r="O9" s="5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="P9" s="5" t="s">
         <v>48</v>
       </c>
       <c r="Q9" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="R9" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="R9" s="5" t="s">
+      <c r="S9" s="5" t="s">
         <v>91</v>
-      </c>
-      <c r="S9" s="5" t="s">
-        <v>92</v>
       </c>
       <c r="T9" s="5" t="s">
         <v>46</v>
       </c>
       <c r="U9" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="V9" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="V9" s="5" t="s">
+      <c r="W9" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="X9" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="Y9" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="W9" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="X9" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="Y9" s="5" t="s">
-        <v>98</v>
-      </c>
       <c r="Z9" s="5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="AA9" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AB9" s="5" t="s">
         <v>46</v>
@@ -2153,16 +2153,16 @@
         <v>30</v>
       </c>
       <c r="AE9" s="5" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="AF9" s="5" t="s">
         <v>49</v>
       </c>
       <c r="AG9" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="AH9" s="5" t="s">
         <v>100</v>
-      </c>
-      <c r="AH9" s="5" t="s">
-        <v>101</v>
       </c>
       <c r="AI9" s="6" t="s">
         <v>32</v>
@@ -2179,16 +2179,16 @@
         <v>4</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="K10" s="5" t="s">
         <v>41</v>
       </c>
       <c r="L10" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="M10" s="5" t="s">
         <v>106</v>
-      </c>
-      <c r="M10" s="5" t="s">
-        <v>107</v>
       </c>
       <c r="N10" s="5" t="s">
         <v>33</v>
@@ -2197,25 +2197,25 @@
         <v>49</v>
       </c>
       <c r="P10" s="5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="Q10" s="5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="R10" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="S10" s="5" t="s">
         <v>103</v>
-      </c>
-      <c r="S10" s="5" t="s">
-        <v>104</v>
       </c>
       <c r="T10" s="5" t="s">
         <v>50</v>
       </c>
       <c r="U10" s="5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="V10" s="5" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="W10" s="5" t="s">
         <v>45</v>
@@ -2224,13 +2224,13 @@
         <v>49</v>
       </c>
       <c r="Y10" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="Z10" s="5" t="s">
         <v>29</v>
       </c>
       <c r="AA10" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="AB10" s="5" t="s">
         <v>50</v>
@@ -2242,10 +2242,10 @@
         <v>36</v>
       </c>
       <c r="AE10" s="5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="AF10" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AG10" s="5" t="s">
         <v>56</v>
@@ -2276,7 +2276,7 @@
         <v>9</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="13" spans="1:35" x14ac:dyDescent="0.3">
@@ -2303,13 +2303,13 @@
     </row>
     <row r="15" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A15" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B15" s="8" t="s">
         <v>6</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="16" spans="1:35" x14ac:dyDescent="0.3">
@@ -2336,13 +2336,13 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B18" s="8" t="s">
         <v>15</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">

</xml_diff>